<commit_message>
update code 05-02-2026 23:00
</commit_message>
<xml_diff>
--- a/dashboard_report.xlsx
+++ b/dashboard_report.xlsx
@@ -415,12 +415,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -454,16 +454,16 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>10500</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>-37.5%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="D2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -474,16 +474,16 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>-50.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="D3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -514,16 +514,16 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>10500</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>-37.5%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="D5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6"/>
@@ -583,43 +583,43 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2600</v>
-      </c>
-    </row>
-    <row r="13"/>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Weekly Sales</t>
-        </is>
-      </c>
-    </row>
+        <v>10500</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Label</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Value</t>
+          <t>Weekly Sales</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>0</v>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Mon</t>
+          <t>Sun</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -629,7 +629,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Tue</t>
+          <t>Mon</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -639,7 +639,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Wed</t>
+          <t>Tue</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -649,7 +649,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Thu</t>
+          <t>Wed</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -659,7 +659,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Fri</t>
+          <t>Thu</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -669,10 +669,20 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="B22" t="n">
+      <c r="B23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -687,11 +697,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
@@ -726,7 +736,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>119449</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -786,7 +796,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>119449</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -858,40 +868,40 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Weekly Sales</t>
-        </is>
-      </c>
-    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>119449</v>
+      </c>
+    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Label</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Value</t>
+          <t>Weekly Sales</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>0</v>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Mon</t>
+          <t>Sun</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -901,7 +911,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Tue</t>
+          <t>Mon</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -911,7 +921,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Wed</t>
+          <t>Tue</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -921,7 +931,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Thu</t>
+          <t>Wed</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -931,7 +941,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Fri</t>
+          <t>Thu</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -941,11 +951,21 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Sat</t>
+          <t>Fri</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>119449</v>
       </c>
     </row>
   </sheetData>
@@ -959,14 +979,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="6" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -984,7 +1004,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1008,7 +1028,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -1047,39 +1067,2439 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ITEM001</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Wahoo Ceviche</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Cold Appetizer</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>7500.00</t>
+        </is>
+      </c>
+    </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>ITEM002</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Lobster Thermidor</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Mains</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>19200.00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>ITEM003</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Margherita</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Pizza</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>9</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>5400.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ITEM004</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>JIM BEAM 1Lt.</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>BOURBON</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>19</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>76000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ITEM005</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>JIM BEAM Per Shot</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>BOURBON</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>12</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>3000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ITEM006</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>JIM BEAM BLACK</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>BOURBON</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>5</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>25000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ITEM007</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Tuna Crudo</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Cold Appetizer</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>17</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>8500.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ITEM008</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Estrella Galicia</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Beers</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>750.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ITEM009</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Heineken</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Beers</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>500.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ITEM010</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>San Mig Apple</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Beers</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>4</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>600.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ITEM011</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>MOET CHANDON BRUT</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>CHAMPAGNE / SPARKLING WINE</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>3</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>31500.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>ITEM012</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>HENESSY VS 750ml</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>COGNAC / BRANDY</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>4</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>34000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ITEM013</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Pinacolada</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Classic Cocktails</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>900.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ITEM014</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Sex On The Beach</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Classic Cocktails</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>600.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ITEM015</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Green Tea</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Coffee &amp; Tea</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>90.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ITEM016</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Mango Lemonade</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Mocktails</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>4</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>1200.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ITEM017</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>SPELLBOUND PINOT NOIR</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>RED WINE</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>6000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>ITEM018</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>MAKERS MARK 750ML</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>BOURBON</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>21</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>157500.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>ITEM019</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Coconut Mousse</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Dessert</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>21</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>6300.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ITEM020</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Split Bill Paid</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>33</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>-298282.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>ITEM021</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Americano</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Coffee &amp; Tea</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>4</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>640.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>ITEM022</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Cafe Latte</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Coffee &amp; Tea</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>10</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2500.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>ITEM023</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Black Tea</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Coffee &amp; Tea</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>3</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>270.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ITEM024</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Calamares</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Crispy Bites</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>12</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>4800.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>ITEM025</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Mexisisig</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Sizzlers</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>9</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>4950.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>ITEM026</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Pulled Beef Sandwich</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Sandwiches, Burgers &amp; Snacks</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>550.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>ITEM027</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Caesar Salad Grande</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Salad &amp; Dips</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>10</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>6000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>ITEM028</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Chirashi Sashimi</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Pizza</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>7</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>5250.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>ITEM029</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Marina Verde Lasagna</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Pasta</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>12</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>8040.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>ITEM030</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Salmon</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Fresh from the Sea</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>2</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>800.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>ITEM031</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>DOM PERIGNON BRUT</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>CHAMPAGNE / SPARKLING WINE</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>45000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>ITEM032</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>VEUVE CLIQUOT BRUT</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>CHAMPAGNE / SPARKLING WINE</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>6</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>75000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>ITEM033</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Pizza Frita Ala Nutella Smores</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Dessert</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>8</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2400.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>ITEM034</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Carbonara Oceanica</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Pasta</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>9</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>5850.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>ITEM035</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Quattro Formaggi Quesadilla</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Sandwiches, Burgers &amp; Snacks</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>5</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>3490.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ITEM036</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Fisherman's pot</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Soup</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>4</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>ITEM037</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Tuna</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Fresh from the Sea</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>6</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>2400.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>ITEM038</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>San Mig Light</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Beers</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>11</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>1650.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>ITEM039</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Amaretto Sour</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Classic Cocktails</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>2</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>600.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>ITEM040</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Port Barton Sunset</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Signature Cocktails</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>10</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>5500.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>ITEM041</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Blue Ocean Mule</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Signature Cocktails</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>7</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>3850.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>ITEM042</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>PATRON REPOSADO 750ML</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>TEQUILA</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>12500.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>ITEM043</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Sizzling Tuna Bites</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Sizzlers</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>3</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>1350.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>ITEM044</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Ragu Alla Bolognese With Parmesan Espuma</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Pasta</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>7</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>4200.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>ITEM045</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Spiced Cinnamon Apple Spritz</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Signature Cocktails</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>3</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>1650.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>ITEM046</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Salmon Poke</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Cold Appetizer</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>10</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>5000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ITEM047</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Angus Ribeye</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Mains</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>5</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>12500.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>ITEM048</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Crispy Pork Belly</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Mains</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>4</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>2400.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>ITEM049</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>San Mig Pale Pilsen</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Beers</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>17</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>2550.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>ITEM050</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Coke Regular</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Sodas &amp; Water</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>2</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>240.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>ITEM051</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>J. WALKER DOUBLE BLACK Per Shot</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>WHISKY/WHISKEY</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>2</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>700.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>ITEM052</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Fruity Daiqueri</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Classic Cocktails</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>3</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>900.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>ITEM053</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Fruity Margarita</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Classic Cocktails</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>14</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>4200.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>ITEM054</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Cosmopolitan</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Classic Cocktails</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>4</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>1200.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>ITEM055</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>fresh Fruit Platter</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Dessert</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>4</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>1200.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>ITEM056</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Mango</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Shakes/Juices</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>4</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>1000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>ITEM057</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>San Mig Pure Malt</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Beers</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>7</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>1750.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>ITEM058</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Prawn Croquettes</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Crispy Bites</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>2</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>800.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>ITEM059</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Pepperoni</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Pizza</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>6</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>4200.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>ITEM060</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Mango Shake</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>1</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>250.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>ITEM061</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Pineapple</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Shakes/Juices</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>1</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>250.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>ITEM062</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Appetizers</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>18</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>414.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>ITEM063</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Espresso</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Coffee &amp; Tea</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>1</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>150.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>ITEM064</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Cafe Mocha</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Coffee &amp; Tea</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>5</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>1250.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>ITEM065</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Rice</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Mains</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>3</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>180.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>ITEM066</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>KAYAKING</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>1</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>500.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>ITEM067</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Smoked Buffalo Wings</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Crispy Bites</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>8</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>3200.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>ITEM068</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Tropicale</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Pizza</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>2</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>1300.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>ITEM069</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Sunset View - C1 - Main Deck</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>1</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>ITEM070</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Front Facade - T18 - Main Deck</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>1</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>ITEM071</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Front Facade - T19 - Main Deck</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>1</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>ITEM072</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Sunset View - C2 - Main Deck</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>1</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>ITEM073</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Sunset View - C3 - Main Deck</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>1</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>ITEM074</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Caipiranha</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Classic Cocktails</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>2</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>600.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>ITEM075</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Ginger-Basil-Cucumber Lemonade</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Mocktails</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>6</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>1800.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>ITEM076</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Bottled Water</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Sodas &amp; Water</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>10</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>1000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>ITEM077</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Coke Zero</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Sodas &amp; Water</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>2</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>240.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>ITEM078</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Sprite</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Sodas &amp; Water</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>9</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>1080.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>ITEM079</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>MAI TAI WD</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Classic Cocktails</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>37</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>11100.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>ITEM080</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Buffet</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Mains</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>37</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>55500.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>ITEM081</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Jacuzzi Couch - C4 - Main Deck</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>2</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>ITEM082</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Jacuzzi Couch - C7 - Main Deck</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>1</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>ITEM083</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Front Facade - T1 - Main Deck</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>1</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>ITEM084</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Daiquiri</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Classic Cocktails</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>2</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>600.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>ITEM085</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>JOSE CUERVO GOLD 1Lt.</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>TEQUILA</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>1</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>5500.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="93"/>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Staff</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
           <t>Rank</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B95" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C95" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D95" t="inlineStr">
         <is>
           <t>Role</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E95" t="inlineStr">
         <is>
           <t>Guests</t>
         </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Armie Rose Rey</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>S001</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Staff</t>
+        </is>
+      </c>
+      <c r="E96" t="n">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Cherry Ann Lumactod</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>S002</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Staff</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Anna Mae Dela Fuente</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>S003</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Staff</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Elaine Dela Cruz</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>S004</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Staff</t>
+        </is>
+      </c>
+      <c r="E99" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Cashier</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>S005</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Staff</t>
+        </is>
+      </c>
+      <c r="E100" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Dimee Dela Cruz</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>S006</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Staff</t>
+        </is>
+      </c>
+      <c r="E101" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Joraly Angeles</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>S007</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Staff</t>
+        </is>
+      </c>
+      <c r="E102" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Joey Elijan</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>S008</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Staff</t>
+        </is>
+      </c>
+      <c r="E103" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Kenneth John Mart Jusos</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>S009</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Staff</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Rexan Gleem Gaid</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>S010</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Staff</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Arjunren Valdez</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>S011</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Staff</t>
+        </is>
+      </c>
+      <c r="E106" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>